<commit_message>
docs: complete CMS and Payment System design
</commit_message>
<xml_diff>
--- a/docs/02. Source Systems/01. Partner App/Partner_App_Data_Dictionary.xlsx
+++ b/docs/02. Source Systems/01. Partner App/Partner_App_Data_Dictionary.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\consumer-finance-analytics-platform\docs\02. Source Systems\01. Partner App\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00625CD3-C849-46E2-8B17-F20C412252ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC619B13-5720-42F6-8E9E-1C6D2B4FCC99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="partner" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="441" uniqueCount="179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="447" uniqueCount="181">
   <si>
     <t>Column</t>
   </si>
@@ -228,15 +228,9 @@
     <t>0912</t>
   </si>
   <si>
-    <t>national_id</t>
-  </si>
-  <si>
     <t>CCCD</t>
   </si>
   <si>
-    <t>001</t>
-  </si>
-  <si>
     <t>date_of_birth</t>
   </si>
   <si>
@@ -384,9 +378,6 @@
     <t>Số điện thoại</t>
   </si>
   <si>
-    <t>Mã quốc gia</t>
-  </si>
-  <si>
     <t>Ngày tháng năm sinh</t>
   </si>
   <si>
@@ -562,6 +553,21 @@
   </si>
   <si>
     <t>PostgreSQL</t>
+  </si>
+  <si>
+    <t>customer_type</t>
+  </si>
+  <si>
+    <t>NEW_TO_BANK,RELOAN</t>
+  </si>
+  <si>
+    <t>RELOAN</t>
+  </si>
+  <si>
+    <t>Phân loại khách hàng</t>
+  </si>
+  <si>
+    <t>citizen_id</t>
   </si>
 </sst>
 </file>
@@ -978,7 +984,7 @@
   <sheetData>
     <row r="1" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="8" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>0</v>
@@ -1013,7 +1019,7 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>10</v>
@@ -1036,7 +1042,7 @@
       </c>
       <c r="I2" s="3"/>
       <c r="J2" s="4" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="K2" s="3" t="s">
         <v>14</v>
@@ -1044,7 +1050,7 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>15</v>
@@ -1068,12 +1074,12 @@
         <v>18</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>19</v>
@@ -1093,12 +1099,12 @@
         <v>21</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>22</v>
@@ -1125,7 +1131,7 @@
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>27</v>
@@ -1154,7 +1160,7 @@
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>32</v>
@@ -1173,7 +1179,7 @@
       </c>
       <c r="I7" s="3"/>
       <c r="J7" s="3" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K7" s="3" t="s">
         <v>35</v>
@@ -1181,7 +1187,7 @@
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>36</v>
@@ -1198,7 +1204,7 @@
       <c r="H8" s="3"/>
       <c r="I8" s="3"/>
       <c r="J8" s="3" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="K8" s="3" t="s">
         <v>38</v>
@@ -1228,7 +1234,7 @@
   <sheetData>
     <row r="1" spans="1:11" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="8" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>0</v>
@@ -1263,7 +1269,7 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="B2" s="5" t="s">
         <v>39</v>
@@ -1287,12 +1293,12 @@
       <c r="I2" s="5"/>
       <c r="J2" s="5"/>
       <c r="K2" s="5" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="B3" s="5" t="s">
         <v>10</v>
@@ -1312,12 +1318,12 @@
       <c r="I3" s="5"/>
       <c r="J3" s="5"/>
       <c r="K3" s="5" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="B4" s="5" t="s">
         <v>41</v>
@@ -1339,12 +1345,12 @@
         <v>42</v>
       </c>
       <c r="K4" s="5" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>43</v>
@@ -1364,12 +1370,12 @@
         <v>44</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="B6" s="5" t="s">
         <v>45</v>
@@ -1391,12 +1397,12 @@
         <v>47</v>
       </c>
       <c r="K6" s="5" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="B7" s="5" t="s">
         <v>48</v>
@@ -1418,12 +1424,12 @@
         <v>50</v>
       </c>
       <c r="K7" s="5" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="B8" s="5" t="s">
         <v>51</v>
@@ -1441,12 +1447,12 @@
       <c r="I8" s="5"/>
       <c r="J8" s="5"/>
       <c r="K8" s="5" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="B9" s="5" t="s">
         <v>53</v>
@@ -1464,12 +1470,12 @@
       <c r="I9" s="5"/>
       <c r="J9" s="5"/>
       <c r="K9" s="5" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="B10" s="5" t="s">
         <v>54</v>
@@ -1498,7 +1504,7 @@
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="B11" s="5" t="s">
         <v>27</v>
@@ -1522,12 +1528,12 @@
         <v>29</v>
       </c>
       <c r="K11" s="5" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="B12" s="5" t="s">
         <v>32</v>
@@ -1552,7 +1558,7 @@
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="B13" s="5" t="s">
         <v>36</v>
@@ -1580,7 +1586,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:K16"/>
+  <dimension ref="A1:K17"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.33203125" customWidth="1"/>
@@ -1597,7 +1603,7 @@
   <sheetData>
     <row r="1" spans="1:11" ht="31.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="8" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>0</v>
@@ -1632,7 +1638,7 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="B2" s="5" t="s">
         <v>61</v>
@@ -1656,12 +1662,12 @@
       <c r="I2" s="5"/>
       <c r="J2" s="5"/>
       <c r="K2" s="5" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="B3" s="5" t="s">
         <v>10</v>
@@ -1681,12 +1687,12 @@
       <c r="I3" s="5"/>
       <c r="J3" s="5"/>
       <c r="K3" s="5" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="B4" s="5" t="s">
         <v>39</v>
@@ -1706,12 +1712,12 @@
       <c r="I4" s="5"/>
       <c r="J4" s="5"/>
       <c r="K4" s="5" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>63</v>
@@ -1731,12 +1737,12 @@
         <v>64</v>
       </c>
       <c r="K5" s="5" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="B6" s="5" t="s">
         <v>65</v>
@@ -1756,15 +1762,15 @@
         <v>66</v>
       </c>
       <c r="K6" s="5" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>67</v>
+        <v>180</v>
       </c>
       <c r="C7" s="5" t="s">
         <v>28</v>
@@ -1777,21 +1783,21 @@
       <c r="G7" s="5"/>
       <c r="H7" s="5"/>
       <c r="I7" s="5" t="s">
-        <v>68</v>
-      </c>
-      <c r="J7" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
+      </c>
+      <c r="J7" s="5">
+        <v>1234567890</v>
       </c>
       <c r="K7" s="5" t="s">
-        <v>119</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C8" s="5" t="s">
         <v>52</v>
@@ -1806,18 +1812,18 @@
       <c r="I8" s="5"/>
       <c r="J8" s="5"/>
       <c r="K8" s="5" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="D9" s="5"/>
       <c r="E9" s="5"/>
@@ -1827,21 +1833,21 @@
       <c r="G9" s="5"/>
       <c r="H9" s="5"/>
       <c r="I9" s="5" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="J9" s="5" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="K9" s="5" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C10" s="5" t="s">
         <v>55</v>
@@ -1857,18 +1863,18 @@
         <v>57</v>
       </c>
       <c r="J10" s="5" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="K10" s="5" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C11" s="5" t="s">
         <v>55</v>
@@ -1881,24 +1887,24 @@
       <c r="G11" s="5"/>
       <c r="H11" s="5"/>
       <c r="I11" s="5" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="J11" s="5" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="K11" s="5" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D12" s="5"/>
       <c r="E12" s="5"/>
@@ -1908,24 +1914,24 @@
       <c r="G12" s="5"/>
       <c r="H12" s="5"/>
       <c r="I12" s="5" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="J12" s="5" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="K12" s="5" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="D13" s="5"/>
       <c r="E13" s="5"/>
@@ -1935,24 +1941,24 @@
       <c r="G13" s="5"/>
       <c r="H13" s="5"/>
       <c r="I13" s="5" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J13" s="5" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="K13" s="5" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>27</v>
+        <v>176</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="D14" s="5"/>
       <c r="E14" s="5"/>
@@ -1960,28 +1966,26 @@
         <v>12</v>
       </c>
       <c r="G14" s="5"/>
-      <c r="H14" s="5" t="s">
-        <v>88</v>
-      </c>
+      <c r="H14" s="5"/>
       <c r="I14" s="5" t="s">
-        <v>89</v>
+        <v>177</v>
       </c>
       <c r="J14" s="5" t="s">
-        <v>88</v>
+        <v>178</v>
       </c>
       <c r="K14" s="5" t="s">
-        <v>135</v>
+        <v>179</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="D15" s="5"/>
       <c r="E15" s="5"/>
@@ -1990,20 +1994,24 @@
       </c>
       <c r="G15" s="5"/>
       <c r="H15" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="I15" s="5"/>
-      <c r="J15" s="5"/>
-      <c r="K15" s="3" t="s">
-        <v>35</v>
+        <v>86</v>
+      </c>
+      <c r="I15" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="J15" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="K15" s="5" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C16" s="5" t="s">
         <v>33</v>
@@ -2011,13 +2019,38 @@
       <c r="D16" s="5"/>
       <c r="E16" s="5"/>
       <c r="F16" s="5" t="s">
-        <v>37</v>
+        <v>12</v>
       </c>
       <c r="G16" s="5"/>
-      <c r="H16" s="5"/>
+      <c r="H16" s="5" t="s">
+        <v>34</v>
+      </c>
       <c r="I16" s="5"/>
       <c r="J16" s="5"/>
       <c r="K16" s="3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A17" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D17" s="5"/>
+      <c r="E17" s="5"/>
+      <c r="F17" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="G17" s="5"/>
+      <c r="H17" s="5"/>
+      <c r="I17" s="5"/>
+      <c r="J17" s="5"/>
+      <c r="K17" s="3" t="s">
         <v>38</v>
       </c>
     </row>
@@ -2045,7 +2078,7 @@
   <sheetData>
     <row r="1" spans="1:11" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="8" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>0</v>
@@ -2080,10 +2113,10 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C2" s="5" t="s">
         <v>11</v>
@@ -2104,12 +2137,12 @@
       <c r="I2" s="5"/>
       <c r="J2" s="5"/>
       <c r="K2" s="1" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="B3" s="5" t="s">
         <v>61</v>
@@ -2119,7 +2152,7 @@
       </c>
       <c r="D3" s="5"/>
       <c r="E3" s="5" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="F3" s="5" t="s">
         <v>12</v>
@@ -2129,18 +2162,18 @@
       <c r="I3" s="5"/>
       <c r="J3" s="5"/>
       <c r="K3" s="1" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="D4" s="5"/>
       <c r="E4" s="5"/>
@@ -2153,18 +2186,18 @@
       <c r="H4" s="5"/>
       <c r="I4" s="5"/>
       <c r="J4" s="5" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C5" s="5" t="s">
         <v>16</v>
@@ -2176,24 +2209,24 @@
       </c>
       <c r="G5" s="5"/>
       <c r="H5" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="J5" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="I5" s="5" t="s">
-        <v>96</v>
-      </c>
-      <c r="J5" s="5" t="s">
-        <v>97</v>
-      </c>
       <c r="K5" s="1" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C6" s="5" t="s">
         <v>33</v>
@@ -2210,18 +2243,18 @@
       <c r="I6" s="5"/>
       <c r="J6" s="5"/>
       <c r="K6" s="1" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="D7" s="5"/>
       <c r="E7" s="5"/>
@@ -2232,18 +2265,18 @@
       <c r="H7" s="5"/>
       <c r="I7" s="5"/>
       <c r="J7" s="5" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="C8" s="5" t="s">
         <v>23</v>
@@ -2257,21 +2290,21 @@
       <c r="H8" s="5"/>
       <c r="I8" s="5"/>
       <c r="J8" s="5" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="K8" s="5" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D9" s="5"/>
       <c r="E9" s="5"/>
@@ -2282,15 +2315,15 @@
       <c r="H9" s="5"/>
       <c r="I9" s="5"/>
       <c r="J9" s="5" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="B10" s="5" t="s">
         <v>32</v>
@@ -2315,7 +2348,7 @@
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="B11" s="5" t="s">
         <v>36</v>
@@ -2361,19 +2394,19 @@
   <sheetData>
     <row r="1" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="7" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>1</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="F1" s="2" t="s">
         <v>6</v>
@@ -2390,37 +2423,37 @@
     </row>
     <row r="2" spans="1:9" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="B2" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="D2" s="5" t="s">
         <v>137</v>
       </c>
-      <c r="C2" s="5" t="s">
-        <v>139</v>
-      </c>
-      <c r="D2" s="5" t="s">
-        <v>140</v>
-      </c>
       <c r="E2" s="5" t="s">
         <v>12</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="G2" s="5"/>
       <c r="H2" s="5" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>61</v>
@@ -2434,93 +2467,93 @@
       <c r="F3" s="5"/>
       <c r="G3" s="5"/>
       <c r="H3" s="5" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="E4" s="5" t="s">
         <v>12</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="G4" s="5"/>
       <c r="H4" s="5" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="E5" s="5" t="s">
         <v>12</v>
       </c>
       <c r="F5" s="5"/>
       <c r="G5" s="6" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="I5" s="5" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="E6" s="5" t="s">
         <v>37</v>
       </c>
       <c r="F6" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>161</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="I6" s="5" t="s">
         <v>163</v>
-      </c>
-      <c r="G6" s="5" t="s">
-        <v>164</v>
-      </c>
-      <c r="H6" s="5" t="s">
-        <v>165</v>
-      </c>
-      <c r="I6" s="5" t="s">
-        <v>166</v>
       </c>
     </row>
   </sheetData>
@@ -2549,19 +2582,19 @@
   <sheetData>
     <row r="1" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="7" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>1</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="F1" s="2" t="s">
         <v>6</v>
@@ -2578,37 +2611,37 @@
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="E2" s="5" t="s">
         <v>12</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="G2" s="5"/>
       <c r="H2" s="5" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>61</v>
@@ -2622,120 +2655,120 @@
       <c r="F3" s="5"/>
       <c r="G3" s="5"/>
       <c r="H3" s="5" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="E4" s="5" t="s">
         <v>12</v>
       </c>
       <c r="F4" s="5"/>
       <c r="G4" s="5" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="C5" s="5" t="s">
         <v>27</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="E5" s="5" t="s">
         <v>12</v>
       </c>
       <c r="F5" s="5"/>
       <c r="G5" s="5" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="I5" s="5" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="E6" s="5" t="s">
         <v>12</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="G6" s="5"/>
       <c r="H6" s="5" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="I6" s="5" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="B7" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="C7" s="5" t="s">
         <v>147</v>
       </c>
-      <c r="C7" s="5" t="s">
-        <v>150</v>
-      </c>
       <c r="D7" s="5" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="E7" s="5" t="s">
         <v>12</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="H7" s="5" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="I7" s="5" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: update data dictionary
</commit_message>
<xml_diff>
--- a/docs/02. Source Systems/01. Partner App/Partner_App_Data_Dictionary.xlsx
+++ b/docs/02. Source Systems/01. Partner App/Partner_App_Data_Dictionary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\consumer-finance-analytics-platform\docs\02. Source Systems\01. Partner App\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC619B13-5720-42F6-8E9E-1C6D2B4FCC99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15434CC8-3276-42C9-86B8-AEC784D9EB1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="partner" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="447" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="452" uniqueCount="183">
   <si>
     <t>Column</t>
   </si>
@@ -568,6 +568,12 @@
   </si>
   <si>
     <t>citizen_id</t>
+  </si>
+  <si>
+    <t>customer_id</t>
+  </si>
+  <si>
+    <t>Mã khách hàng</t>
   </si>
 </sst>
 </file>
@@ -1586,7 +1592,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:K17"/>
+  <dimension ref="A1:K18"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.33203125" customWidth="1"/>
@@ -1705,7 +1711,7 @@
         <v>62</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>12</v>
+        <v>37</v>
       </c>
       <c r="G4" s="5"/>
       <c r="H4" s="5"/>
@@ -1720,10 +1726,10 @@
         <v>175</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>63</v>
+        <v>181</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="D5" s="5"/>
       <c r="E5" s="5"/>
@@ -1733,22 +1739,20 @@
       <c r="G5" s="5"/>
       <c r="H5" s="5"/>
       <c r="I5" s="5"/>
-      <c r="J5" s="5" t="s">
-        <v>64</v>
-      </c>
+      <c r="J5" s="5"/>
       <c r="K5" s="5" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>175</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="D6" s="5"/>
       <c r="E6" s="5"/>
@@ -1759,18 +1763,18 @@
       <c r="H6" s="5"/>
       <c r="I6" s="5"/>
       <c r="J6" s="5" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="K6" s="5" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>175</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>180</v>
+        <v>65</v>
       </c>
       <c r="C7" s="5" t="s">
         <v>28</v>
@@ -1782,14 +1786,12 @@
       </c>
       <c r="G7" s="5"/>
       <c r="H7" s="5"/>
-      <c r="I7" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="J7" s="5">
-        <v>1234567890</v>
+      <c r="I7" s="5"/>
+      <c r="J7" s="5" t="s">
+        <v>66</v>
       </c>
       <c r="K7" s="5" t="s">
-        <v>14</v>
+        <v>116</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.3">
@@ -1797,10 +1799,10 @@
         <v>175</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>68</v>
+        <v>180</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>52</v>
+        <v>28</v>
       </c>
       <c r="D8" s="5"/>
       <c r="E8" s="5"/>
@@ -1809,10 +1811,14 @@
       </c>
       <c r="G8" s="5"/>
       <c r="H8" s="5"/>
-      <c r="I8" s="5"/>
-      <c r="J8" s="5"/>
+      <c r="I8" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="J8" s="5">
+        <v>1234567890</v>
+      </c>
       <c r="K8" s="5" t="s">
-        <v>117</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.3">
@@ -1820,10 +1826,10 @@
         <v>175</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>70</v>
+        <v>52</v>
       </c>
       <c r="D9" s="5"/>
       <c r="E9" s="5"/>
@@ -1832,14 +1838,10 @@
       </c>
       <c r="G9" s="5"/>
       <c r="H9" s="5"/>
-      <c r="I9" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="J9" s="5" t="s">
-        <v>72</v>
-      </c>
+      <c r="I9" s="5"/>
+      <c r="J9" s="5"/>
       <c r="K9" s="5" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.3">
@@ -1847,10 +1849,10 @@
         <v>175</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>55</v>
+        <v>70</v>
       </c>
       <c r="D10" s="5"/>
       <c r="E10" s="5"/>
@@ -1860,13 +1862,13 @@
       <c r="G10" s="5"/>
       <c r="H10" s="5"/>
       <c r="I10" s="5" t="s">
-        <v>57</v>
+        <v>71</v>
       </c>
       <c r="J10" s="5" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="K10" s="5" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.3">
@@ -1874,7 +1876,7 @@
         <v>175</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C11" s="5" t="s">
         <v>55</v>
@@ -1887,13 +1889,13 @@
       <c r="G11" s="5"/>
       <c r="H11" s="5"/>
       <c r="I11" s="5" t="s">
-        <v>76</v>
+        <v>57</v>
       </c>
       <c r="J11" s="5" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="K11" s="5" t="s">
-        <v>129</v>
+        <v>119</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.3">
@@ -1901,10 +1903,10 @@
         <v>175</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>79</v>
+        <v>55</v>
       </c>
       <c r="D12" s="5"/>
       <c r="E12" s="5"/>
@@ -1914,13 +1916,13 @@
       <c r="G12" s="5"/>
       <c r="H12" s="5"/>
       <c r="I12" s="5" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="J12" s="5" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="K12" s="5" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.3">
@@ -1928,26 +1930,26 @@
         <v>175</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="D13" s="5"/>
       <c r="E13" s="5"/>
       <c r="F13" s="5" t="s">
-        <v>37</v>
+        <v>12</v>
       </c>
       <c r="G13" s="5"/>
       <c r="H13" s="5"/>
       <c r="I13" s="5" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="J13" s="5" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="K13" s="5" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.3">
@@ -1955,26 +1957,26 @@
         <v>175</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>176</v>
+        <v>82</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>28</v>
+        <v>83</v>
       </c>
       <c r="D14" s="5"/>
       <c r="E14" s="5"/>
       <c r="F14" s="5" t="s">
-        <v>12</v>
+        <v>37</v>
       </c>
       <c r="G14" s="5"/>
       <c r="H14" s="5"/>
       <c r="I14" s="5" t="s">
-        <v>177</v>
+        <v>84</v>
       </c>
       <c r="J14" s="5" t="s">
-        <v>178</v>
+        <v>85</v>
       </c>
       <c r="K14" s="5" t="s">
-        <v>179</v>
+        <v>131</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.3">
@@ -1982,10 +1984,10 @@
         <v>175</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>27</v>
+        <v>176</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="D15" s="5"/>
       <c r="E15" s="5"/>
@@ -1993,17 +1995,15 @@
         <v>12</v>
       </c>
       <c r="G15" s="5"/>
-      <c r="H15" s="5" t="s">
-        <v>86</v>
-      </c>
+      <c r="H15" s="5"/>
       <c r="I15" s="5" t="s">
-        <v>87</v>
+        <v>177</v>
       </c>
       <c r="J15" s="5" t="s">
-        <v>86</v>
+        <v>178</v>
       </c>
       <c r="K15" s="5" t="s">
-        <v>132</v>
+        <v>179</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.3">
@@ -2011,10 +2011,10 @@
         <v>175</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="D16" s="5"/>
       <c r="E16" s="5"/>
@@ -2023,12 +2023,16 @@
       </c>
       <c r="G16" s="5"/>
       <c r="H16" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="I16" s="5"/>
-      <c r="J16" s="5"/>
-      <c r="K16" s="3" t="s">
-        <v>35</v>
+        <v>86</v>
+      </c>
+      <c r="I16" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="J16" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="K16" s="5" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.3">
@@ -2036,7 +2040,7 @@
         <v>175</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C17" s="5" t="s">
         <v>33</v>
@@ -2044,13 +2048,38 @@
       <c r="D17" s="5"/>
       <c r="E17" s="5"/>
       <c r="F17" s="5" t="s">
-        <v>37</v>
+        <v>12</v>
       </c>
       <c r="G17" s="5"/>
-      <c r="H17" s="5"/>
+      <c r="H17" s="5" t="s">
+        <v>34</v>
+      </c>
       <c r="I17" s="5"/>
       <c r="J17" s="5"/>
       <c r="K17" s="3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A18" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D18" s="5"/>
+      <c r="E18" s="5"/>
+      <c r="F18" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="G18" s="5"/>
+      <c r="H18" s="5"/>
+      <c r="I18" s="5"/>
+      <c r="J18" s="5"/>
+      <c r="K18" s="3" t="s">
         <v>38</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: add database DDL structure
</commit_message>
<xml_diff>
--- a/docs/02. Source Systems/01. Partner App/Partner_App_Data_Dictionary.xlsx
+++ b/docs/02. Source Systems/01. Partner App/Partner_App_Data_Dictionary.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\consumer-finance-analytics-platform\docs\02. Source Systems\01. Partner App\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15434CC8-3276-42C9-86B8-AEC784D9EB1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E35089C8-4DAB-4C10-B2FC-17A1FA7EAEC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="452" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="473" uniqueCount="193">
   <si>
     <t>Column</t>
   </si>
@@ -574,6 +574,36 @@
   </si>
   <si>
     <t>Mã khách hàng</t>
+  </si>
+  <si>
+    <t>product_group</t>
+  </si>
+  <si>
+    <t>product_code</t>
+  </si>
+  <si>
+    <t>CASH</t>
+  </si>
+  <si>
+    <t>CASH_LOAN,CREDIT_CARD</t>
+  </si>
+  <si>
+    <t>CASH_LOAN</t>
+  </si>
+  <si>
+    <t>Mã sản phẩm vay</t>
+  </si>
+  <si>
+    <t>Loại sản phẩm vay</t>
+  </si>
+  <si>
+    <t>LOAN,CARD</t>
+  </si>
+  <si>
+    <t>requested_credit_limit</t>
+  </si>
+  <si>
+    <t>Hạn mức thẻ</t>
   </si>
 </sst>
 </file>
@@ -1592,11 +1622,11 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:K18"/>
+  <dimension ref="A1:K21"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.33203125" customWidth="1"/>
-    <col min="2" max="2" width="16.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.5546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="13.21875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="5" customWidth="1"/>
     <col min="5" max="5" width="19.77734375" bestFit="1" customWidth="1"/>
@@ -1734,7 +1764,7 @@
       <c r="D5" s="5"/>
       <c r="E5" s="5"/>
       <c r="F5" s="5" t="s">
-        <v>12</v>
+        <v>37</v>
       </c>
       <c r="G5" s="5"/>
       <c r="H5" s="5"/>
@@ -1911,7 +1941,7 @@
       <c r="D12" s="5"/>
       <c r="E12" s="5"/>
       <c r="F12" s="5" t="s">
-        <v>12</v>
+        <v>37</v>
       </c>
       <c r="G12" s="5"/>
       <c r="H12" s="5"/>
@@ -1938,7 +1968,7 @@
       <c r="D13" s="5"/>
       <c r="E13" s="5"/>
       <c r="F13" s="5" t="s">
-        <v>12</v>
+        <v>37</v>
       </c>
       <c r="G13" s="5"/>
       <c r="H13" s="5"/>
@@ -1957,10 +1987,10 @@
         <v>175</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>82</v>
+        <v>191</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>83</v>
+        <v>55</v>
       </c>
       <c r="D14" s="5"/>
       <c r="E14" s="5"/>
@@ -1970,13 +2000,13 @@
       <c r="G14" s="5"/>
       <c r="H14" s="5"/>
       <c r="I14" s="5" t="s">
-        <v>84</v>
+        <v>57</v>
       </c>
       <c r="J14" s="5" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="K14" s="5" t="s">
-        <v>131</v>
+        <v>192</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.3">
@@ -1984,26 +2014,26 @@
         <v>175</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>176</v>
+        <v>82</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>28</v>
+        <v>83</v>
       </c>
       <c r="D15" s="5"/>
       <c r="E15" s="5"/>
       <c r="F15" s="5" t="s">
-        <v>12</v>
+        <v>37</v>
       </c>
       <c r="G15" s="5"/>
       <c r="H15" s="5"/>
       <c r="I15" s="5" t="s">
-        <v>177</v>
+        <v>84</v>
       </c>
       <c r="J15" s="5" t="s">
-        <v>178</v>
+        <v>85</v>
       </c>
       <c r="K15" s="5" t="s">
-        <v>179</v>
+        <v>131</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.3">
@@ -2011,10 +2041,10 @@
         <v>175</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>27</v>
+        <v>176</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="D16" s="5"/>
       <c r="E16" s="5"/>
@@ -2022,17 +2052,15 @@
         <v>12</v>
       </c>
       <c r="G16" s="5"/>
-      <c r="H16" s="5" t="s">
-        <v>86</v>
-      </c>
+      <c r="H16" s="5"/>
       <c r="I16" s="5" t="s">
-        <v>87</v>
+        <v>177</v>
       </c>
       <c r="J16" s="5" t="s">
-        <v>86</v>
+        <v>178</v>
       </c>
       <c r="K16" s="5" t="s">
-        <v>132</v>
+        <v>179</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.3">
@@ -2040,10 +2068,10 @@
         <v>175</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="D17" s="5"/>
       <c r="E17" s="5"/>
@@ -2052,12 +2080,16 @@
       </c>
       <c r="G17" s="5"/>
       <c r="H17" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="I17" s="5"/>
-      <c r="J17" s="5"/>
-      <c r="K17" s="3" t="s">
-        <v>35</v>
+        <v>86</v>
+      </c>
+      <c r="I17" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="J17" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="K17" s="5" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.3">
@@ -2065,21 +2097,100 @@
         <v>175</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>36</v>
+        <v>183</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="D18" s="5"/>
       <c r="E18" s="5"/>
       <c r="F18" s="5" t="s">
-        <v>37</v>
+        <v>12</v>
       </c>
       <c r="G18" s="5"/>
       <c r="H18" s="5"/>
-      <c r="I18" s="5"/>
-      <c r="J18" s="5"/>
-      <c r="K18" s="3" t="s">
+      <c r="I18" s="5" t="s">
+        <v>190</v>
+      </c>
+      <c r="J18" s="5" t="s">
+        <v>185</v>
+      </c>
+      <c r="K18" s="5" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A19" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D19" s="5"/>
+      <c r="E19" s="5"/>
+      <c r="F19" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G19" s="5"/>
+      <c r="H19" s="5"/>
+      <c r="I19" s="5" t="s">
+        <v>186</v>
+      </c>
+      <c r="J19" s="5" t="s">
+        <v>187</v>
+      </c>
+      <c r="K19" s="5" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A20" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D20" s="5"/>
+      <c r="E20" s="5"/>
+      <c r="F20" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G20" s="5"/>
+      <c r="H20" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="I20" s="5"/>
+      <c r="J20" s="5"/>
+      <c r="K20" s="3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A21" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="B21" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D21" s="5"/>
+      <c r="E21" s="5"/>
+      <c r="F21" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="G21" s="5"/>
+      <c r="H21" s="5"/>
+      <c r="I21" s="5"/>
+      <c r="J21" s="5"/>
+      <c r="K21" s="3" t="s">
         <v>38</v>
       </c>
     </row>

</xml_diff>